<commit_message>
Sync planning SharePoint : S39
</commit_message>
<xml_diff>
--- a/Plannings 2026 S39.xlsx
+++ b/Plannings 2026 S39.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38550F53-A7D0-45C7-9442-056190286F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{38550F53-A7D0-45C7-9442-056190286F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A06EF1BD-7F7B-483F-A397-D5C858F621BE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6120,7 +6120,7 @@
       <c r="A46" s="20"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
-      <c r="D46" s="3" t="s">
+      <c r="D46" s="39" t="s">
         <v>47</v>
       </c>
       <c r="E46" s="2"/>
@@ -6132,7 +6132,7 @@
       <c r="A47" s="22"/>
       <c r="B47" s="24"/>
       <c r="C47" s="24"/>
-      <c r="D47" s="24" t="s">
+      <c r="D47" s="38" t="s">
         <v>75</v>
       </c>
       <c r="E47" s="24"/>
@@ -6274,7 +6274,7 @@
       </c>
       <c r="B56" s="18"/>
       <c r="C56" s="18"/>
-      <c r="D56" s="18" t="s">
+      <c r="D56" s="45" t="s">
         <v>18</v>
       </c>
       <c r="E56" s="18"/>
@@ -6288,7 +6288,7 @@
       <c r="A57" s="20"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
-      <c r="D57" s="2" t="s">
+      <c r="D57" s="46" t="s">
         <v>19</v>
       </c>
       <c r="E57" s="2"/>
@@ -6302,7 +6302,7 @@
       <c r="A58" s="20"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
+      <c r="D58" s="46"/>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
       <c r="G58" s="47" t="s">
@@ -6314,7 +6314,7 @@
       <c r="A59" s="22"/>
       <c r="B59" s="24"/>
       <c r="C59" s="24"/>
-      <c r="D59" s="24"/>
+      <c r="D59" s="48"/>
       <c r="E59" s="24"/>
       <c r="F59" s="24"/>
       <c r="G59" s="48" t="s">
@@ -7543,13 +7543,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18701F86-DB93-445C-953C-8C414000BBB7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86DDF764-0B5A-44B5-AB40-319194553184}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52AB36C8-F5FF-481C-A64F-24BA079B375D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35247376-8E7F-4853-B503-C64174BE633A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBA61D21-BDB7-44B7-A672-E6D0A824BB75}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2C474F2-04FB-4666-8D32-FACE7FBF4504}"/>
 </file>
</xml_diff>